<commit_message>
fix(portfolio): corriger tickers/refPrices depuis PDF Coris + BICB + fallback refPrice
https://claude.ai/code/session_01Cczp8DqGBrELUNJJw8JJfc
</commit_message>
<xml_diff>
--- a/BRVM_Portefeuille_Tiaho_09062026.xlsx
+++ b/BRVM_Portefeuille_Tiaho_09062026.xlsx
@@ -1245,7 +1245,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>SOGC</t>
+          <t>SOGB</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>SIVC</t>
+          <t>LACI</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>SDSC</t>
+          <t>SDCC</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>BOA CI</t>
+          <t>BOA Côte d'Ivoire</t>
         </is>
       </c>
       <c r="D16" s="30" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>CBIBF</t>
+          <t>CBBF</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="E31" s="44" t="inlineStr">
         <is>
-          <t>Gain &gt;80% (ETIT, CBIBF, NSBC) — envisager une prise de bénéfices partielle</t>
+          <t>Gain &gt;80% (ETIT, CBBF, NSBC) — envisager une prise de bénéfices partielle</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>CBIBF</t>
+          <t>CBBF</t>
         </is>
       </c>
       <c r="C4" s="21" t="inlineStr">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>SDSC</t>
+          <t>SDCC</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>BOA CI</t>
+          <t>BOA Côte d'Ivoire</t>
         </is>
       </c>
       <c r="D13" s="62" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>SOGC</t>
+          <t>SOGB</t>
         </is>
       </c>
       <c r="C16" s="21" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>SIVC</t>
+          <t>LACI</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">

</xml_diff>

<commit_message>
fix(portfolio): corriger le ticker Air Liquide CI — LACI → SIVC
LACI n'est pas un ticker BRVM valide. Le ticker officiel est SIVC
(Erium Côte d'Ivoire, ex-Air Liquide CI), déjà utilisé dans database.py.

https://claude.ai/code/session_01Cczp8DqGBrELUNJJw8JJfc
</commit_message>
<xml_diff>
--- a/BRVM_Portefeuille_Tiaho_09062026.xlsx
+++ b/BRVM_Portefeuille_Tiaho_09062026.xlsx
@@ -1525,12 +1525,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>LACI</t>
+          <t>SIVC</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Air Liquide CI</t>
+          <t>Erium CI (ex-Air Liquide)</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -3456,12 +3456,12 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>LACI</t>
+          <t>SIVC</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>Air Liquide CI</t>
+          <t>Erium CI (ex-Air Liquide)</t>
         </is>
       </c>
       <c r="D18" s="64" t="inlineStr">

</xml_diff>

<commit_message>
fix(portfolio): corriger le ticker AGL CI (ex-Bolloré) — SDCC → SDSC
Régression introduite par une correction précédente qui avait renommé
SDSC en SDCC en pensant corriger une faute de frappe. Or SDCC et SDSC
sont deux sociétés BRVM distinctes (cf. database.py) :
  - SDCC = SODECI (distribution d'eau)
  - SDSC = AGL CI — Africa Global Logistics (ex-Bolloré Transport &
    Logistique), qui correspond à la position réelle du portefeuille.

https://claude.ai/code/session_01Cczp8DqGBrELUNJJw8JJfc
</commit_message>
<xml_diff>
--- a/BRVM_Portefeuille_Tiaho_09062026.xlsx
+++ b/BRVM_Portefeuille_Tiaho_09062026.xlsx
@@ -1875,12 +1875,12 @@
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>SDCC</t>
+          <t>SDSC</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
         <is>
-          <t>Bolloré Transport CI</t>
+          <t>AGL CI (ex-Bolloré)</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
@@ -3155,12 +3155,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>SDCC</t>
+          <t>SDSC</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Bolloré Transport CI</t>
+          <t>AGL CI (ex-Bolloré)</t>
         </is>
       </c>
       <c r="D11" s="62" t="inlineStr">

</xml_diff>

<commit_message>
fix(portfolio): corriger le coût moyen pondéré BOAM (4 achats distincts)
7 @ 4980 + 11 @ 4905 + 7 @ 4690 + 5 @ 4675 = 30 titres @ 4 834 F
(au lieu de 4 890 F). P&L : -4.2% au lieu de -5.3%.

https://claude.ai/code/session_01Cczp8DqGBrELUNJJw8JJfc
</commit_message>
<xml_diff>
--- a/BRVM_Portefeuille_Tiaho_09062026.xlsx
+++ b/BRVM_Portefeuille_Tiaho_09062026.xlsx
@@ -2172,7 +2172,7 @@
         <v>30</v>
       </c>
       <c r="F19" s="23" t="n">
-        <v>4890</v>
+        <v>4834</v>
       </c>
       <c r="G19" s="24">
         <f>E19*F19</f>
@@ -3685,13 +3685,13 @@
         </is>
       </c>
       <c r="E23" s="65" t="n">
-        <v>-0.05316973415132924</v>
+        <v>-0.04220107571369466</v>
       </c>
       <c r="F23" s="66" t="n">
-        <v>-7800</v>
+        <v>-6120</v>
       </c>
       <c r="G23" s="54" t="n">
-        <v>4890</v>
+        <v>4834</v>
       </c>
       <c r="H23" s="55" t="n">
         <v>4630</v>
@@ -3711,14 +3711,14 @@
     <row r="25">
       <c r="A25" s="69" t="inlineStr">
         <is>
-          <t>TOTAL PORTEFEUILLE — Coût : 7,026,271 F  ·  Valeur : 9,316,395 F</t>
+          <t>TOTAL PORTEFEUILLE — Coût : 7,024,591 F  ·  Valeur : 9,316,395 F</t>
         </is>
       </c>
       <c r="E25" s="70" t="n">
-        <v>0.3259373286342073</v>
+        <v>0.3262544395823188</v>
       </c>
       <c r="F25" s="71" t="n">
-        <v>2290124</v>
+        <v>2291804</v>
       </c>
     </row>
   </sheetData>

</xml_diff>